<commit_message>
research: expand public phase 3 evidence
</commit_message>
<xml_diff>
--- a/research/phase-3/Phase_3_B2B_Buyer_List.xlsx
+++ b/research/phase-3/Phase_3_B2B_Buyer_List.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Buyers" sheetId="1" r:id="Ra44ebe6f3c574c82"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Buyers" sheetId="1" r:id="R137f6e37b1fd4730"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -337,44 +337,48 @@
         <x:v>Peru</x:v>
       </x:c>
       <x:c r="B2" s="4" t="str">
-        <x:v>Zongshen Peru</x:v>
+        <x:v>Zonsen Peru / Grupo Cayman</x:v>
       </x:c>
       <x:c r="C2" s="4" t="str">
         <x:v>Brand/service channel</x:v>
       </x:c>
       <x:c r="D2" s="4" t="str">
-        <x:v>Zongshen</x:v>
+        <x:v>Zonsen</x:v>
       </x:c>
       <x:c r="E2" s="4" t="str">
-        <x:v>Motorcycles; service</x:v>
+        <x:v>Motorcycles; service; parts</x:v>
       </x:c>
       <x:c r="F2" s="4" t="str">
-        <x:v>Wholesale claim</x:v>
+        <x:v>Wholesale and parts routes</x:v>
       </x:c>
       <x:c r="G2" s="4" t="str">
-        <x:v>https://zongshenperu.com/garantia-post-venta/</x:v>
-      </x:c>
-      <x:c r="H2" s="4" t="str"/>
+        <x:v>https://zonsenperu.com.pe/garantia-post-venta/</x:v>
+      </x:c>
+      <x:c r="H2" s="4" t="str">
+        <x:v>Lewis Gonzalez</x:v>
+      </x:c>
       <x:c r="I2" s="4" t="str"/>
-      <x:c r="J2" s="4" t="str"/>
+      <x:c r="J2" s="4" t="str">
+        <x:v>929412843</x:v>
+      </x:c>
       <x:c r="K2" s="4" t="str"/>
       <x:c r="L2" s="4" t="str">
         <x:v>Peru</x:v>
       </x:c>
       <x:c r="M2" s="4" t="str">
-        <x:v>Public business route</x:v>
+        <x:v>Public phone</x:v>
       </x:c>
       <x:c r="N2" s="4" t="str">
-        <x:v>P3-P01</x:v>
+        <x:v>P3-P05</x:v>
       </x:c>
       <x:c r="O2" s="4" t="str">
-        <x:v>Channel mapping</x:v>
+        <x:v>Chinese-brand channel</x:v>
       </x:c>
       <x:c r="P2" s="4" t="str">
         <x:v>Complete-engine demand unproven</x:v>
       </x:c>
       <x:c r="Q2" s="4" t="str">
-        <x:v>Medium</x:v>
+        <x:v>High</x:v>
       </x:c>
       <x:c r="R2" s="4" t="str">
         <x:v>NOT CONTACTED</x:v>
@@ -385,22 +389,22 @@
         <x:v>Peru</x:v>
       </x:c>
       <x:c r="B3" s="4" t="str">
-        <x:v>Maquirsa</x:v>
+        <x:v>Zongshen Peru</x:v>
       </x:c>
       <x:c r="C3" s="4" t="str">
-        <x:v>Parts wholesaler</x:v>
+        <x:v>Brand/service channel</x:v>
       </x:c>
       <x:c r="D3" s="4" t="str">
-        <x:v>Lifan; Zongshen</x:v>
+        <x:v>Zongshen</x:v>
       </x:c>
       <x:c r="E3" s="4" t="str">
-        <x:v>Parts</x:v>
+        <x:v>Motorcycles; service</x:v>
       </x:c>
       <x:c r="F3" s="4" t="str">
-        <x:v>Parts channel</x:v>
+        <x:v>Wholesale claim</x:v>
       </x:c>
       <x:c r="G3" s="4" t="str">
-        <x:v>https://maquirsa.com/contacto/</x:v>
+        <x:v>https://zongshenperu.com/garantia-post-venta/</x:v>
       </x:c>
       <x:c r="H3" s="4" t="str"/>
       <x:c r="I3" s="4" t="str"/>
@@ -413,13 +417,13 @@
         <x:v>Public business route</x:v>
       </x:c>
       <x:c r="N3" s="4" t="str">
-        <x:v>P3-P02</x:v>
+        <x:v>P3-P01</x:v>
       </x:c>
       <x:c r="O3" s="4" t="str">
-        <x:v>Parts-pack validation</x:v>
+        <x:v>Channel mapping</x:v>
       </x:c>
       <x:c r="P3" s="4" t="str">
-        <x:v>Parts is not engine demand</x:v>
+        <x:v>Complete-engine demand unproven</x:v>
       </x:c>
       <x:c r="Q3" s="4" t="str">
         <x:v>Medium</x:v>
@@ -430,48 +434,44 @@
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="4" t="str">
-        <x:v>Ecuador</x:v>
+        <x:v>Peru</x:v>
       </x:c>
       <x:c r="B4" s="4" t="str">
-        <x:v>Shineray Ecuador</x:v>
+        <x:v>Maquirsa</x:v>
       </x:c>
       <x:c r="C4" s="4" t="str">
-        <x:v>Importer/distributor</x:v>
+        <x:v>Parts wholesaler</x:v>
       </x:c>
       <x:c r="D4" s="4" t="str">
-        <x:v>Shineray</x:v>
+        <x:v>Lifan; Zongshen</x:v>
       </x:c>
       <x:c r="E4" s="4" t="str">
-        <x:v>Motorcycles; distributor network</x:v>
+        <x:v>Parts</x:v>
       </x:c>
       <x:c r="F4" s="4" t="str">
-        <x:v>Official distributor</x:v>
+        <x:v>Parts channel</x:v>
       </x:c>
       <x:c r="G4" s="4" t="str">
-        <x:v>https://www.shineray.com.ec/distribuidores</x:v>
+        <x:v>https://maquirsa.com/contacto/</x:v>
       </x:c>
       <x:c r="H4" s="4" t="str"/>
-      <x:c r="I4" s="4" t="str">
-        <x:v>info@shineray.com.ec</x:v>
-      </x:c>
-      <x:c r="J4" s="4" t="str">
-        <x:v>1-800-744627</x:v>
-      </x:c>
+      <x:c r="I4" s="4" t="str"/>
+      <x:c r="J4" s="4" t="str"/>
       <x:c r="K4" s="4" t="str"/>
       <x:c r="L4" s="4" t="str">
-        <x:v>Guayaquil</x:v>
+        <x:v>Peru</x:v>
       </x:c>
       <x:c r="M4" s="4" t="str">
-        <x:v>Public email/phone</x:v>
+        <x:v>Public business route</x:v>
       </x:c>
       <x:c r="N4" s="4" t="str">
-        <x:v>P3-E01</x:v>
+        <x:v>P3-P02</x:v>
       </x:c>
       <x:c r="O4" s="4" t="str">
-        <x:v>Chinese-brand channel</x:v>
+        <x:v>Parts-pack validation</x:v>
       </x:c>
       <x:c r="P4" s="4" t="str">
-        <x:v>Engine procurement unproven</x:v>
+        <x:v>Parts is not engine demand</x:v>
       </x:c>
       <x:c r="Q4" s="4" t="str">
         <x:v>Medium</x:v>
@@ -482,44 +482,48 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="4" t="str">
-        <x:v>Ecuador</x:v>
+        <x:v>Peru</x:v>
       </x:c>
       <x:c r="B5" s="4" t="str">
-        <x:v>Zongshen Ecuador</x:v>
+        <x:v>Corporacion Mabel</x:v>
       </x:c>
       <x:c r="C5" s="4" t="str">
-        <x:v>Brand/dealer</x:v>
+        <x:v>Importer/wholesaler</x:v>
       </x:c>
       <x:c r="D5" s="4" t="str">
-        <x:v>Zongshen</x:v>
+        <x:v>Various</x:v>
       </x:c>
       <x:c r="E5" s="4" t="str">
-        <x:v>Motorcycles</x:v>
+        <x:v>Motorcycle; mototaxi; cargo-motorcycle parts</x:v>
       </x:c>
       <x:c r="F5" s="4" t="str">
-        <x:v>Official contact</x:v>
+        <x:v>Importer and wholesale claim</x:v>
       </x:c>
       <x:c r="G5" s="4" t="str">
-        <x:v>https://zongshenecuador.com/contacto</x:v>
+        <x:v>https://corporacionmabel.pe/</x:v>
       </x:c>
       <x:c r="H5" s="4" t="str"/>
-      <x:c r="I5" s="4" t="str"/>
-      <x:c r="J5" s="4" t="str"/>
+      <x:c r="I5" s="4" t="str">
+        <x:v>ventas@corporacionmabel.pe</x:v>
+      </x:c>
+      <x:c r="J5" s="4" t="str">
+        <x:v>965030502</x:v>
+      </x:c>
       <x:c r="K5" s="4" t="str"/>
       <x:c r="L5" s="4" t="str">
-        <x:v>Cuenca</x:v>
+        <x:v>Cusco</x:v>
       </x:c>
       <x:c r="M5" s="4" t="str">
-        <x:v>Public address</x:v>
+        <x:v>Public email/phone</x:v>
       </x:c>
       <x:c r="N5" s="4" t="str">
-        <x:v>P3-E02</x:v>
+        <x:v>P3-P04</x:v>
       </x:c>
       <x:c r="O5" s="4" t="str">
-        <x:v>Channel mapping</x:v>
+        <x:v>Cargo/mototaxi channel</x:v>
       </x:c>
       <x:c r="P5" s="4" t="str">
-        <x:v>Engine demand unproven</x:v>
+        <x:v>Parts-only evidence</x:v>
       </x:c>
       <x:c r="Q5" s="4" t="str">
         <x:v>Medium</x:v>
@@ -530,44 +534,46 @@
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="4" t="str">
-        <x:v>Tanzania</x:v>
+        <x:v>Peru</x:v>
       </x:c>
       <x:c r="B6" s="4" t="str">
-        <x:v>Guta Trading (T) Ltd</x:v>
+        <x:v>JP Motorcycles</x:v>
       </x:c>
       <x:c r="C6" s="4" t="str">
-        <x:v>Cargo 3R/parts dealer</x:v>
+        <x:v>Importer/distributor</x:v>
       </x:c>
       <x:c r="D6" s="4" t="str">
-        <x:v>Lifan</x:v>
+        <x:v>Various</x:v>
       </x:c>
       <x:c r="E6" s="4" t="str">
-        <x:v>Cargo tricycles; spares</x:v>
+        <x:v>Motorcycles; parts</x:v>
       </x:c>
       <x:c r="F6" s="4" t="str">
-        <x:v>Company claim</x:v>
+        <x:v>Import/distribution and wholesale claim</x:v>
       </x:c>
       <x:c r="G6" s="4" t="str">
-        <x:v>https://guta.co.tz/</x:v>
+        <x:v>https://jpmotorcycles.pe/la-empresa/</x:v>
       </x:c>
       <x:c r="H6" s="4" t="str"/>
       <x:c r="I6" s="4" t="str"/>
-      <x:c r="J6" s="4" t="str"/>
+      <x:c r="J6" s="4" t="str">
+        <x:v>951788512</x:v>
+      </x:c>
       <x:c r="K6" s="4" t="str"/>
       <x:c r="L6" s="4" t="str">
-        <x:v>Dar es Salaam</x:v>
+        <x:v>Peru</x:v>
       </x:c>
       <x:c r="M6" s="4" t="str">
-        <x:v>Public company contact</x:v>
+        <x:v>Public phone</x:v>
       </x:c>
       <x:c r="N6" s="4" t="str">
-        <x:v>P3-T01</x:v>
+        <x:v>P3-P06</x:v>
       </x:c>
       <x:c r="O6" s="4" t="str">
-        <x:v>Cargo/parts validation</x:v>
+        <x:v>Wholesale channel</x:v>
       </x:c>
       <x:c r="P6" s="4" t="str">
-        <x:v>Engine demand unproven</x:v>
+        <x:v>Complete-engine demand unproven</x:v>
       </x:c>
       <x:c r="Q6" s="4" t="str">
         <x:v>Medium</x:v>
@@ -578,47 +584,47 @@
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="4" t="str">
-        <x:v>Tanzania</x:v>
+        <x:v>Peru</x:v>
       </x:c>
       <x:c r="B7" s="4" t="str">
-        <x:v>Sinoray Mobility Solutions</x:v>
+        <x:v>Repuestos Delivery</x:v>
       </x:c>
       <x:c r="C7" s="4" t="str">
-        <x:v>Motorcycle/parts channel</x:v>
+        <x:v>Parts importer</x:v>
       </x:c>
       <x:c r="D7" s="4" t="str">
-        <x:v>Sinoray</x:v>
+        <x:v>Various</x:v>
       </x:c>
       <x:c r="E7" s="4" t="str">
-        <x:v>Motorcycles; parts</x:v>
+        <x:v>Motorcycle; mototaxi; cargo parts</x:v>
       </x:c>
       <x:c r="F7" s="4" t="str">
-        <x:v>Company claim</x:v>
+        <x:v>Importer claim</x:v>
       </x:c>
       <x:c r="G7" s="4" t="str">
-        <x:v>https://www.sinoraymotor.com/</x:v>
+        <x:v>https://repuestosdelivery.pe/index.html</x:v>
       </x:c>
       <x:c r="H7" s="4" t="str"/>
       <x:c r="I7" s="4" t="str"/>
       <x:c r="J7" s="4" t="str"/>
       <x:c r="K7" s="4" t="str"/>
       <x:c r="L7" s="4" t="str">
-        <x:v>Tanzania</x:v>
+        <x:v>Peru</x:v>
       </x:c>
       <x:c r="M7" s="4" t="str">
-        <x:v>Public company contact</x:v>
+        <x:v>Public company route</x:v>
       </x:c>
       <x:c r="N7" s="4" t="str">
-        <x:v>P3-T02</x:v>
+        <x:v>P3-P07</x:v>
       </x:c>
       <x:c r="O7" s="4" t="str">
-        <x:v>Channel mapping</x:v>
+        <x:v>Parts-pack validation</x:v>
       </x:c>
       <x:c r="P7" s="4" t="str">
-        <x:v>Engine demand unproven</x:v>
+        <x:v>Parts-only; Indian platforms excluded</x:v>
       </x:c>
       <x:c r="Q7" s="4" t="str">
-        <x:v>Medium</x:v>
+        <x:v>Low</x:v>
       </x:c>
       <x:c r="R7" s="4" t="str">
         <x:v>NOT CONTACTED</x:v>
@@ -626,47 +632,47 @@
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="4" t="str">
-        <x:v>Uzbekistan</x:v>
+        <x:v>Peru</x:v>
       </x:c>
       <x:c r="B8" s="4" t="str">
-        <x:v>Bikeland</x:v>
+        <x:v>Motos Racing</x:v>
       </x:c>
       <x:c r="C8" s="4" t="str">
-        <x:v>Retailer/service</x:v>
+        <x:v>Brand/parts channel</x:v>
       </x:c>
       <x:c r="D8" s="4" t="str">
-        <x:v>Lifan; Zongshen</x:v>
+        <x:v>Zongshen</x:v>
       </x:c>
       <x:c r="E8" s="4" t="str">
-        <x:v>Motorcycles; tricycles; engines; parts</x:v>
+        <x:v>Motorcycles; imported parts</x:v>
       </x:c>
       <x:c r="F8" s="4" t="str">
-        <x:v>Website listing</x:v>
+        <x:v>Zongshen representation claim</x:v>
       </x:c>
       <x:c r="G8" s="4" t="str">
-        <x:v>https://www.bikeland.uz/</x:v>
+        <x:v>https://motosracing.pe/tiendas/tienda-san-juan-de-miraflores</x:v>
       </x:c>
       <x:c r="H8" s="4" t="str"/>
       <x:c r="I8" s="4" t="str"/>
       <x:c r="J8" s="4" t="str"/>
       <x:c r="K8" s="4" t="str"/>
       <x:c r="L8" s="4" t="str">
-        <x:v>Uzbekistan</x:v>
+        <x:v>Lima</x:v>
       </x:c>
       <x:c r="M8" s="4" t="str">
         <x:v>Public company route</x:v>
       </x:c>
       <x:c r="N8" s="4" t="str">
-        <x:v>P3-U01</x:v>
+        <x:v>P3-P08</x:v>
       </x:c>
       <x:c r="O8" s="4" t="str">
-        <x:v>Accelerated validation</x:v>
+        <x:v>Brand/channel mapping</x:v>
       </x:c>
       <x:c r="P8" s="4" t="str">
-        <x:v>Retailer not national wholesaler</x:v>
+        <x:v>Complete-engine demand unproven</x:v>
       </x:c>
       <x:c r="Q8" s="4" t="str">
-        <x:v>Medium</x:v>
+        <x:v>Low</x:v>
       </x:c>
       <x:c r="R8" s="4" t="str">
         <x:v>NOT CONTACTED</x:v>
@@ -674,47 +680,45 @@
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="4" t="str">
-        <x:v>Russia</x:v>
+        <x:v>Peru</x:v>
       </x:c>
       <x:c r="B9" s="4" t="str">
-        <x:v>Loncin Russia</x:v>
+        <x:v>Autocar Repuestos</x:v>
       </x:c>
       <x:c r="C9" s="4" t="str">
-        <x:v>Official representative</x:v>
+        <x:v>Tricycle-related channel candidate</x:v>
       </x:c>
       <x:c r="D9" s="4" t="str">
-        <x:v>Loncin</x:v>
+        <x:v>Mixed incl. excluded Indian brands</x:v>
       </x:c>
       <x:c r="E9" s="4" t="str">
-        <x:v>Motorcycles/parts</x:v>
+        <x:v>Parts/vehicles</x:v>
       </x:c>
       <x:c r="F9" s="4" t="str">
-        <x:v>Representative page</x:v>
-      </x:c>
-      <x:c r="G9" s="4" t="str">
-        <x:v>https://loncin.pro/company</x:v>
-      </x:c>
+        <x:v>Secondary candidate only</x:v>
+      </x:c>
+      <x:c r="G9" s="4" t="str"/>
       <x:c r="H9" s="4" t="str"/>
       <x:c r="I9" s="4" t="str"/>
       <x:c r="J9" s="4" t="str"/>
       <x:c r="K9" s="4" t="str"/>
       <x:c r="L9" s="4" t="str">
-        <x:v>Russia</x:v>
+        <x:v>Peru</x:v>
       </x:c>
       <x:c r="M9" s="4" t="str">
-        <x:v>Public company route</x:v>
+        <x:v>NOT VERIFIED</x:v>
       </x:c>
       <x:c r="N9" s="4" t="str">
-        <x:v>P3-R01</x:v>
+        <x:v>P3-P07</x:v>
       </x:c>
       <x:c r="O9" s="4" t="str">
-        <x:v>Distributor mapping</x:v>
+        <x:v>Requires independent verification</x:v>
       </x:c>
       <x:c r="P9" s="4" t="str">
-        <x:v>Compliance unresolved</x:v>
+        <x:v>Mixed platforms; no direct source</x:v>
       </x:c>
       <x:c r="Q9" s="4" t="str">
-        <x:v>Medium</x:v>
+        <x:v>Low</x:v>
       </x:c>
       <x:c r="R9" s="4" t="str">
         <x:v>NOT CONTACTED</x:v>
@@ -722,49 +726,1553 @@
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="4" t="str">
-        <x:v>Russia</x:v>
+        <x:v>Peru</x:v>
       </x:c>
       <x:c r="B10" s="4" t="str">
-        <x:v>Lifan Russia</x:v>
+        <x:v>Lifan Peru channel</x:v>
       </x:c>
       <x:c r="C10" s="4" t="str">
-        <x:v>Official representative</x:v>
+        <x:v>Brand-channel candidate</x:v>
       </x:c>
       <x:c r="D10" s="4" t="str">
         <x:v>Lifan</x:v>
       </x:c>
       <x:c r="E10" s="4" t="str">
-        <x:v>Motorcycles/parts</x:v>
+        <x:v>Motorcycles/tricycles</x:v>
       </x:c>
       <x:c r="F10" s="4" t="str">
-        <x:v>Representative page</x:v>
-      </x:c>
-      <x:c r="G10" s="4" t="str">
-        <x:v>https://lifan-moto.ru/</x:v>
-      </x:c>
+        <x:v>Government platform signal only</x:v>
+      </x:c>
+      <x:c r="G10" s="4" t="str"/>
       <x:c r="H10" s="4" t="str"/>
       <x:c r="I10" s="4" t="str"/>
       <x:c r="J10" s="4" t="str"/>
       <x:c r="K10" s="4" t="str"/>
       <x:c r="L10" s="4" t="str">
+        <x:v>Peru</x:v>
+      </x:c>
+      <x:c r="M10" s="4" t="str">
+        <x:v>NOT VERIFIED</x:v>
+      </x:c>
+      <x:c r="N10" s="4" t="str">
+        <x:v>P3-P03</x:v>
+      </x:c>
+      <x:c r="O10" s="4" t="str">
+        <x:v>Platform mapping</x:v>
+      </x:c>
+      <x:c r="P10" s="4" t="str">
+        <x:v>No public buyer route recorded</x:v>
+      </x:c>
+      <x:c r="Q10" s="4" t="str">
+        <x:v>Low</x:v>
+      </x:c>
+      <x:c r="R10" s="4" t="str">
+        <x:v>NOT CONTACTED</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="4" t="str">
+        <x:v>Peru</x:v>
+      </x:c>
+      <x:c r="B11" s="4" t="str">
+        <x:v>Independent cargo-motorcycle assembler</x:v>
+      </x:c>
+      <x:c r="C11" s="4" t="str">
+        <x:v>Assembler candidate</x:v>
+      </x:c>
+      <x:c r="D11" s="4" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="E11" s="4" t="str">
+        <x:v>Cargo motorcycles</x:v>
+      </x:c>
+      <x:c r="F11" s="4" t="str">
+        <x:v>Research target only</x:v>
+      </x:c>
+      <x:c r="G11" s="4" t="str"/>
+      <x:c r="H11" s="4" t="str"/>
+      <x:c r="I11" s="4" t="str"/>
+      <x:c r="J11" s="4" t="str"/>
+      <x:c r="K11" s="4" t="str"/>
+      <x:c r="L11" s="4" t="str">
+        <x:v>Peru</x:v>
+      </x:c>
+      <x:c r="M11" s="4" t="str">
+        <x:v>NOT VERIFIED</x:v>
+      </x:c>
+      <x:c r="N11" s="4" t="str">
+        <x:v>P3-P04</x:v>
+      </x:c>
+      <x:c r="O11" s="4" t="str">
+        <x:v>Validate mixed load</x:v>
+      </x:c>
+      <x:c r="P11" s="4" t="str">
+        <x:v>No named entity evidence</x:v>
+      </x:c>
+      <x:c r="Q11" s="4" t="str">
+        <x:v>Low</x:v>
+      </x:c>
+      <x:c r="R11" s="4" t="str">
+        <x:v>NOT CONTACTED</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="4" t="str">
+        <x:v>Ecuador</x:v>
+      </x:c>
+      <x:c r="B12" s="4" t="str">
+        <x:v>Shineray Ecuador</x:v>
+      </x:c>
+      <x:c r="C12" s="4" t="str">
+        <x:v>Importer/distributor</x:v>
+      </x:c>
+      <x:c r="D12" s="4" t="str">
+        <x:v>Shineray</x:v>
+      </x:c>
+      <x:c r="E12" s="4" t="str">
+        <x:v>Motorcycles; distributor network</x:v>
+      </x:c>
+      <x:c r="F12" s="4" t="str">
+        <x:v>Official distributor</x:v>
+      </x:c>
+      <x:c r="G12" s="4" t="str">
+        <x:v>https://www.shineray.com.ec/distribuidores</x:v>
+      </x:c>
+      <x:c r="H12" s="4" t="str"/>
+      <x:c r="I12" s="4" t="str">
+        <x:v>info@shineray.com.ec</x:v>
+      </x:c>
+      <x:c r="J12" s="4" t="str">
+        <x:v>1-800-744627</x:v>
+      </x:c>
+      <x:c r="K12" s="4" t="str"/>
+      <x:c r="L12" s="4" t="str">
+        <x:v>Guayaquil</x:v>
+      </x:c>
+      <x:c r="M12" s="4" t="str">
+        <x:v>Public email/phone</x:v>
+      </x:c>
+      <x:c r="N12" s="4" t="str">
+        <x:v>P3-E01</x:v>
+      </x:c>
+      <x:c r="O12" s="4" t="str">
+        <x:v>Chinese-brand channel</x:v>
+      </x:c>
+      <x:c r="P12" s="4" t="str">
+        <x:v>Engine procurement unproven</x:v>
+      </x:c>
+      <x:c r="Q12" s="4" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="R12" s="4" t="str">
+        <x:v>NOT CONTACTED</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="4" t="str">
+        <x:v>Ecuador</x:v>
+      </x:c>
+      <x:c r="B13" s="4" t="str">
+        <x:v>Zongshen Ecuador</x:v>
+      </x:c>
+      <x:c r="C13" s="4" t="str">
+        <x:v>Brand/dealer</x:v>
+      </x:c>
+      <x:c r="D13" s="4" t="str">
+        <x:v>Zongshen</x:v>
+      </x:c>
+      <x:c r="E13" s="4" t="str">
+        <x:v>Motorcycles</x:v>
+      </x:c>
+      <x:c r="F13" s="4" t="str">
+        <x:v>Official contact</x:v>
+      </x:c>
+      <x:c r="G13" s="4" t="str">
+        <x:v>https://zongshenecuador.com/contacto</x:v>
+      </x:c>
+      <x:c r="H13" s="4" t="str"/>
+      <x:c r="I13" s="4" t="str"/>
+      <x:c r="J13" s="4" t="str"/>
+      <x:c r="K13" s="4" t="str"/>
+      <x:c r="L13" s="4" t="str">
+        <x:v>Cuenca</x:v>
+      </x:c>
+      <x:c r="M13" s="4" t="str">
+        <x:v>Public address</x:v>
+      </x:c>
+      <x:c r="N13" s="4" t="str">
+        <x:v>P3-E02</x:v>
+      </x:c>
+      <x:c r="O13" s="4" t="str">
+        <x:v>Channel mapping</x:v>
+      </x:c>
+      <x:c r="P13" s="4" t="str">
+        <x:v>Engine demand unproven</x:v>
+      </x:c>
+      <x:c r="Q13" s="4" t="str">
+        <x:v>Medium</x:v>
+      </x:c>
+      <x:c r="R13" s="4" t="str">
+        <x:v>NOT CONTACTED</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="4" t="str">
+        <x:v>Ecuador</x:v>
+      </x:c>
+      <x:c r="B14" s="4" t="str">
+        <x:v>Motoindustria S.A.</x:v>
+      </x:c>
+      <x:c r="C14" s="4" t="str">
+        <x:v>Manufacturer</x:v>
+      </x:c>
+      <x:c r="D14" s="4" t="str">
+        <x:v>TUKO</x:v>
+      </x:c>
+      <x:c r="E14" s="4" t="str">
+        <x:v>Motorcycles</x:v>
+      </x:c>
+      <x:c r="F14" s="4" t="str">
+        <x:v>AEADE listing</x:v>
+      </x:c>
+      <x:c r="G14" s="4" t="str">
+        <x:v>https://www.aeade.net/afiliados/</x:v>
+      </x:c>
+      <x:c r="H14" s="4" t="str"/>
+      <x:c r="I14" s="4" t="str"/>
+      <x:c r="J14" s="4" t="str">
+        <x:v>042811343</x:v>
+      </x:c>
+      <x:c r="K14" s="4" t="str"/>
+      <x:c r="L14" s="4" t="str">
+        <x:v>Guayaquil</x:v>
+      </x:c>
+      <x:c r="M14" s="4" t="str">
+        <x:v>Public phone</x:v>
+      </x:c>
+      <x:c r="N14" s="4" t="str">
+        <x:v>P3-E04</x:v>
+      </x:c>
+      <x:c r="O14" s="4" t="str">
+        <x:v>Assembly/manufacturer validation</x:v>
+      </x:c>
+      <x:c r="P14" s="4" t="str">
+        <x:v>Engine procurement unproven</x:v>
+      </x:c>
+      <x:c r="Q14" s="4" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="R14" s="4" t="str">
+        <x:v>NOT CONTACTED</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="4" t="str">
+        <x:v>Ecuador</x:v>
+      </x:c>
+      <x:c r="B15" s="4" t="str">
+        <x:v>Unnomotors S.A. / Motor1</x:v>
+      </x:c>
+      <x:c r="C15" s="4" t="str">
+        <x:v>Motorcycle commercialiser</x:v>
+      </x:c>
+      <x:c r="D15" s="4" t="str">
+        <x:v>Motor1</x:v>
+      </x:c>
+      <x:c r="E15" s="4" t="str">
+        <x:v>Motorcycles</x:v>
+      </x:c>
+      <x:c r="F15" s="4" t="str">
+        <x:v>AEADE listing</x:v>
+      </x:c>
+      <x:c r="G15" s="4" t="str">
+        <x:v>https://www.aeade.net/afiliados/</x:v>
+      </x:c>
+      <x:c r="H15" s="4" t="str"/>
+      <x:c r="I15" s="4" t="str"/>
+      <x:c r="J15" s="4" t="str"/>
+      <x:c r="K15" s="4" t="str"/>
+      <x:c r="L15" s="4" t="str">
+        <x:v>Cuenca</x:v>
+      </x:c>
+      <x:c r="M15" s="4" t="str">
+        <x:v>Association-listed route</x:v>
+      </x:c>
+      <x:c r="N15" s="4" t="str">
+        <x:v>P3-E04</x:v>
+      </x:c>
+      <x:c r="O15" s="4" t="str">
+        <x:v>Channel mapping</x:v>
+      </x:c>
+      <x:c r="P15" s="4" t="str">
+        <x:v>Procurement role unverified</x:v>
+      </x:c>
+      <x:c r="Q15" s="4" t="str">
+        <x:v>Medium</x:v>
+      </x:c>
+      <x:c r="R15" s="4" t="str">
+        <x:v>NOT CONTACTED</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="4" t="str">
+        <x:v>Ecuador</x:v>
+      </x:c>
+      <x:c r="B16" s="4" t="str">
+        <x:v>Almacenes Juan Eljuri</x:v>
+      </x:c>
+      <x:c r="C16" s="4" t="str">
+        <x:v>Motorcycle commercialiser</x:v>
+      </x:c>
+      <x:c r="D16" s="4" t="str">
+        <x:v>Various</x:v>
+      </x:c>
+      <x:c r="E16" s="4" t="str">
+        <x:v>Motorcycles</x:v>
+      </x:c>
+      <x:c r="F16" s="4" t="str">
+        <x:v>AEADE listing</x:v>
+      </x:c>
+      <x:c r="G16" s="4" t="str">
+        <x:v>https://www.aeade.net/afiliados/</x:v>
+      </x:c>
+      <x:c r="H16" s="4" t="str"/>
+      <x:c r="I16" s="4" t="str"/>
+      <x:c r="J16" s="4" t="str"/>
+      <x:c r="K16" s="4" t="str"/>
+      <x:c r="L16" s="4" t="str">
+        <x:v>Ecuador</x:v>
+      </x:c>
+      <x:c r="M16" s="4" t="str">
+        <x:v>Association-listed route</x:v>
+      </x:c>
+      <x:c r="N16" s="4" t="str">
+        <x:v>P3-E04</x:v>
+      </x:c>
+      <x:c r="O16" s="4" t="str">
+        <x:v>Channel mapping</x:v>
+      </x:c>
+      <x:c r="P16" s="4" t="str">
+        <x:v>Procurement role unverified</x:v>
+      </x:c>
+      <x:c r="Q16" s="4" t="str">
+        <x:v>Medium</x:v>
+      </x:c>
+      <x:c r="R16" s="4" t="str">
+        <x:v>NOT CONTACTED</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="4" t="str">
+        <x:v>Ecuador</x:v>
+      </x:c>
+      <x:c r="B17" s="4" t="str">
+        <x:v>Moto Concept</x:v>
+      </x:c>
+      <x:c r="C17" s="4" t="str">
+        <x:v>Motorcycle commercialiser</x:v>
+      </x:c>
+      <x:c r="D17" s="4" t="str">
+        <x:v>Various</x:v>
+      </x:c>
+      <x:c r="E17" s="4" t="str">
+        <x:v>Motorcycles</x:v>
+      </x:c>
+      <x:c r="F17" s="4" t="str">
+        <x:v>AEADE listing</x:v>
+      </x:c>
+      <x:c r="G17" s="4" t="str">
+        <x:v>https://www.aeade.net/afiliados/</x:v>
+      </x:c>
+      <x:c r="H17" s="4" t="str"/>
+      <x:c r="I17" s="4" t="str"/>
+      <x:c r="J17" s="4" t="str"/>
+      <x:c r="K17" s="4" t="str"/>
+      <x:c r="L17" s="4" t="str">
+        <x:v>Ecuador</x:v>
+      </x:c>
+      <x:c r="M17" s="4" t="str">
+        <x:v>Association-listed route</x:v>
+      </x:c>
+      <x:c r="N17" s="4" t="str">
+        <x:v>P3-E04</x:v>
+      </x:c>
+      <x:c r="O17" s="4" t="str">
+        <x:v>Channel mapping</x:v>
+      </x:c>
+      <x:c r="P17" s="4" t="str">
+        <x:v>Procurement role unverified</x:v>
+      </x:c>
+      <x:c r="Q17" s="4" t="str">
+        <x:v>Low</x:v>
+      </x:c>
+      <x:c r="R17" s="4" t="str">
+        <x:v>NOT CONTACTED</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="4" t="str">
+        <x:v>Ecuador</x:v>
+      </x:c>
+      <x:c r="B18" s="4" t="str">
+        <x:v>Comandato</x:v>
+      </x:c>
+      <x:c r="C18" s="4" t="str">
+        <x:v>Motorcycle commercialiser</x:v>
+      </x:c>
+      <x:c r="D18" s="4" t="str">
+        <x:v>Various</x:v>
+      </x:c>
+      <x:c r="E18" s="4" t="str">
+        <x:v>Motorcycles</x:v>
+      </x:c>
+      <x:c r="F18" s="4" t="str">
+        <x:v>AEADE listing</x:v>
+      </x:c>
+      <x:c r="G18" s="4" t="str">
+        <x:v>https://www.aeade.net/afiliados/</x:v>
+      </x:c>
+      <x:c r="H18" s="4" t="str"/>
+      <x:c r="I18" s="4" t="str"/>
+      <x:c r="J18" s="4" t="str"/>
+      <x:c r="K18" s="4" t="str"/>
+      <x:c r="L18" s="4" t="str">
+        <x:v>Ecuador</x:v>
+      </x:c>
+      <x:c r="M18" s="4" t="str">
+        <x:v>Association-listed route</x:v>
+      </x:c>
+      <x:c r="N18" s="4" t="str">
+        <x:v>P3-E04</x:v>
+      </x:c>
+      <x:c r="O18" s="4" t="str">
+        <x:v>Channel mapping</x:v>
+      </x:c>
+      <x:c r="P18" s="4" t="str">
+        <x:v>Procurement role unverified</x:v>
+      </x:c>
+      <x:c r="Q18" s="4" t="str">
+        <x:v>Low</x:v>
+      </x:c>
+      <x:c r="R18" s="4" t="str">
+        <x:v>NOT CONTACTED</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="4" t="str">
+        <x:v>Ecuador</x:v>
+      </x:c>
+      <x:c r="B19" s="4" t="str">
+        <x:v>Indumot</x:v>
+      </x:c>
+      <x:c r="C19" s="4" t="str">
+        <x:v>Motorcycle commercialiser</x:v>
+      </x:c>
+      <x:c r="D19" s="4" t="str">
+        <x:v>Various</x:v>
+      </x:c>
+      <x:c r="E19" s="4" t="str">
+        <x:v>Motorcycles</x:v>
+      </x:c>
+      <x:c r="F19" s="4" t="str">
+        <x:v>AEADE listing</x:v>
+      </x:c>
+      <x:c r="G19" s="4" t="str">
+        <x:v>https://www.aeade.net/afiliados/</x:v>
+      </x:c>
+      <x:c r="H19" s="4" t="str"/>
+      <x:c r="I19" s="4" t="str"/>
+      <x:c r="J19" s="4" t="str"/>
+      <x:c r="K19" s="4" t="str"/>
+      <x:c r="L19" s="4" t="str">
+        <x:v>Ecuador</x:v>
+      </x:c>
+      <x:c r="M19" s="4" t="str">
+        <x:v>Association-listed route</x:v>
+      </x:c>
+      <x:c r="N19" s="4" t="str">
+        <x:v>P3-E04</x:v>
+      </x:c>
+      <x:c r="O19" s="4" t="str">
+        <x:v>Channel mapping</x:v>
+      </x:c>
+      <x:c r="P19" s="4" t="str">
+        <x:v>Procurement role unverified</x:v>
+      </x:c>
+      <x:c r="Q19" s="4" t="str">
+        <x:v>Low</x:v>
+      </x:c>
+      <x:c r="R19" s="4" t="str">
+        <x:v>NOT CONTACTED</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="4" t="str">
+        <x:v>Ecuador</x:v>
+      </x:c>
+      <x:c r="B20" s="4" t="str">
+        <x:v>Galardi El Inca</x:v>
+      </x:c>
+      <x:c r="C20" s="4" t="str">
+        <x:v>Brand channel</x:v>
+      </x:c>
+      <x:c r="D20" s="4" t="str">
+        <x:v>Loncin; Shineray</x:v>
+      </x:c>
+      <x:c r="E20" s="4" t="str">
+        <x:v>Motorcycles</x:v>
+      </x:c>
+      <x:c r="F20" s="4" t="str">
+        <x:v>Company brand listing</x:v>
+      </x:c>
+      <x:c r="G20" s="4" t="str">
+        <x:v>https://galardielinca.com/</x:v>
+      </x:c>
+      <x:c r="H20" s="4" t="str"/>
+      <x:c r="I20" s="4" t="str"/>
+      <x:c r="J20" s="4" t="str"/>
+      <x:c r="K20" s="4" t="str"/>
+      <x:c r="L20" s="4" t="str">
+        <x:v>Ecuador</x:v>
+      </x:c>
+      <x:c r="M20" s="4" t="str">
+        <x:v>Public company route</x:v>
+      </x:c>
+      <x:c r="N20" s="4" t="str">
+        <x:v>P3-E05</x:v>
+      </x:c>
+      <x:c r="O20" s="4" t="str">
+        <x:v>Chinese-brand channel</x:v>
+      </x:c>
+      <x:c r="P20" s="4" t="str">
+        <x:v>Complete-engine demand unproven</x:v>
+      </x:c>
+      <x:c r="Q20" s="4" t="str">
+        <x:v>Medium</x:v>
+      </x:c>
+      <x:c r="R20" s="4" t="str">
+        <x:v>NOT CONTACTED</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="4" t="str">
+        <x:v>Ecuador</x:v>
+      </x:c>
+      <x:c r="B21" s="4" t="str">
+        <x:v>Almacenes Anderson</x:v>
+      </x:c>
+      <x:c r="C21" s="4" t="str">
+        <x:v>Dealer/retail channel</x:v>
+      </x:c>
+      <x:c r="D21" s="4" t="str">
+        <x:v>Shineray; Loncin</x:v>
+      </x:c>
+      <x:c r="E21" s="4" t="str">
+        <x:v>Motorcycles</x:v>
+      </x:c>
+      <x:c r="F21" s="4" t="str">
+        <x:v>Company brand listing</x:v>
+      </x:c>
+      <x:c r="G21" s="4" t="str">
+        <x:v>https://almacenesanderson.com/</x:v>
+      </x:c>
+      <x:c r="H21" s="4" t="str"/>
+      <x:c r="I21" s="4" t="str"/>
+      <x:c r="J21" s="4" t="str"/>
+      <x:c r="K21" s="4" t="str"/>
+      <x:c r="L21" s="4" t="str">
+        <x:v>Ecuador</x:v>
+      </x:c>
+      <x:c r="M21" s="4" t="str">
+        <x:v>Public company route</x:v>
+      </x:c>
+      <x:c r="N21" s="4" t="str">
+        <x:v>P3-E06</x:v>
+      </x:c>
+      <x:c r="O21" s="4" t="str">
+        <x:v>Channel mapping</x:v>
+      </x:c>
+      <x:c r="P21" s="4" t="str">
+        <x:v>Dealer is not buyer proof</x:v>
+      </x:c>
+      <x:c r="Q21" s="4" t="str">
+        <x:v>Low</x:v>
+      </x:c>
+      <x:c r="R21" s="4" t="str">
+        <x:v>NOT CONTACTED</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="4" t="str">
+        <x:v>Tanzania</x:v>
+      </x:c>
+      <x:c r="B22" s="4" t="str">
+        <x:v>Guta Trading (T) Ltd</x:v>
+      </x:c>
+      <x:c r="C22" s="4" t="str">
+        <x:v>Cargo 3R/parts dealer</x:v>
+      </x:c>
+      <x:c r="D22" s="4" t="str">
+        <x:v>Lifan</x:v>
+      </x:c>
+      <x:c r="E22" s="4" t="str">
+        <x:v>Cargo tricycles; spares</x:v>
+      </x:c>
+      <x:c r="F22" s="4" t="str">
+        <x:v>Company claim</x:v>
+      </x:c>
+      <x:c r="G22" s="4" t="str">
+        <x:v>https://guta.co.tz/</x:v>
+      </x:c>
+      <x:c r="H22" s="4" t="str"/>
+      <x:c r="I22" s="4" t="str">
+        <x:v>info@guta.co.tz</x:v>
+      </x:c>
+      <x:c r="J22" s="4" t="str">
+        <x:v>+255752369000</x:v>
+      </x:c>
+      <x:c r="K22" s="4" t="str"/>
+      <x:c r="L22" s="4" t="str">
+        <x:v>Dar es Salaam</x:v>
+      </x:c>
+      <x:c r="M22" s="4" t="str">
+        <x:v>Public email/phone</x:v>
+      </x:c>
+      <x:c r="N22" s="4" t="str">
+        <x:v>P3-T01</x:v>
+      </x:c>
+      <x:c r="O22" s="4" t="str">
+        <x:v>Cargo/parts validation</x:v>
+      </x:c>
+      <x:c r="P22" s="4" t="str">
+        <x:v>Engine demand unproven</x:v>
+      </x:c>
+      <x:c r="Q22" s="4" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="R22" s="4" t="str">
+        <x:v>NOT CONTACTED</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="4" t="str">
+        <x:v>Tanzania</x:v>
+      </x:c>
+      <x:c r="B23" s="4" t="str">
+        <x:v>Sinoray Mobility Solutions</x:v>
+      </x:c>
+      <x:c r="C23" s="4" t="str">
+        <x:v>Motorcycle/parts channel</x:v>
+      </x:c>
+      <x:c r="D23" s="4" t="str">
+        <x:v>Sinoray</x:v>
+      </x:c>
+      <x:c r="E23" s="4" t="str">
+        <x:v>Motorcycles; parts</x:v>
+      </x:c>
+      <x:c r="F23" s="4" t="str">
+        <x:v>Company claim</x:v>
+      </x:c>
+      <x:c r="G23" s="4" t="str">
+        <x:v>https://www.sinoraymotor.com/</x:v>
+      </x:c>
+      <x:c r="H23" s="4" t="str"/>
+      <x:c r="I23" s="4" t="str"/>
+      <x:c r="J23" s="4" t="str">
+        <x:v>+255652333355</x:v>
+      </x:c>
+      <x:c r="K23" s="4" t="str"/>
+      <x:c r="L23" s="4" t="str">
+        <x:v>Tanzania</x:v>
+      </x:c>
+      <x:c r="M23" s="4" t="str">
+        <x:v>Public phone</x:v>
+      </x:c>
+      <x:c r="N23" s="4" t="str">
+        <x:v>P3-T05</x:v>
+      </x:c>
+      <x:c r="O23" s="4" t="str">
+        <x:v>Channel mapping</x:v>
+      </x:c>
+      <x:c r="P23" s="4" t="str">
+        <x:v>Engine demand unproven</x:v>
+      </x:c>
+      <x:c r="Q23" s="4" t="str">
+        <x:v>Medium</x:v>
+      </x:c>
+      <x:c r="R23" s="4" t="str">
+        <x:v>NOT CONTACTED</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="4" t="str">
+        <x:v>Tanzania</x:v>
+      </x:c>
+      <x:c r="B24" s="4" t="str">
+        <x:v>Fenghao Technology Company Limited</x:v>
+      </x:c>
+      <x:c r="C24" s="4" t="str">
+        <x:v>CKD beneficiary candidate</x:v>
+      </x:c>
+      <x:c r="D24" s="4" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="E24" s="4" t="str">
+        <x:v>Motorcycle/tricycle CKD</x:v>
+      </x:c>
+      <x:c r="F24" s="4" t="str">
+        <x:v>EAC duty-remission listing</x:v>
+      </x:c>
+      <x:c r="G24" s="4" t="str">
+        <x:v>https://www.eac.int/documents?controller=download&amp;file=6c5739ac-842c-43bc-96be-1cd168ed415f&amp;name=EAC+Vol+AT+1+NO+29+SEPTEMBER+2025.pdf&amp;task=download.file</x:v>
+      </x:c>
+      <x:c r="H24" s="4" t="str"/>
+      <x:c r="I24" s="4" t="str"/>
+      <x:c r="J24" s="4" t="str"/>
+      <x:c r="K24" s="4" t="str"/>
+      <x:c r="L24" s="4" t="str">
+        <x:v>Tanzania</x:v>
+      </x:c>
+      <x:c r="M24" s="4" t="str">
+        <x:v>NOT VERIFIED</x:v>
+      </x:c>
+      <x:c r="N24" s="4" t="str">
+        <x:v>P3-T04</x:v>
+      </x:c>
+      <x:c r="O24" s="4" t="str">
+        <x:v>Assembler/CKD validation</x:v>
+      </x:c>
+      <x:c r="P24" s="4" t="str">
+        <x:v>No public contact or engine fit verified</x:v>
+      </x:c>
+      <x:c r="Q24" s="4" t="str">
+        <x:v>Medium</x:v>
+      </x:c>
+      <x:c r="R24" s="4" t="str">
+        <x:v>NOT CONTACTED</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="4" t="str">
+        <x:v>Tanzania</x:v>
+      </x:c>
+      <x:c r="B25" s="4" t="str">
+        <x:v>Munib Enterprise</x:v>
+      </x:c>
+      <x:c r="C25" s="4" t="str">
+        <x:v>CKD beneficiary candidate</x:v>
+      </x:c>
+      <x:c r="D25" s="4" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="E25" s="4" t="str">
+        <x:v>Motorcycle/tricycle CKD</x:v>
+      </x:c>
+      <x:c r="F25" s="4" t="str">
+        <x:v>EAC duty-remission listing</x:v>
+      </x:c>
+      <x:c r="G25" s="4" t="str">
+        <x:v>https://www.eac.int/documents?controller=download&amp;file=6c5739ac-842c-43bc-96be-1cd168ed415f&amp;name=EAC+Vol+AT+1+NO+29+SEPTEMBER+2025.pdf&amp;task=download.file</x:v>
+      </x:c>
+      <x:c r="H25" s="4" t="str"/>
+      <x:c r="I25" s="4" t="str"/>
+      <x:c r="J25" s="4" t="str"/>
+      <x:c r="K25" s="4" t="str"/>
+      <x:c r="L25" s="4" t="str">
+        <x:v>Tanzania</x:v>
+      </x:c>
+      <x:c r="M25" s="4" t="str">
+        <x:v>NOT VERIFIED</x:v>
+      </x:c>
+      <x:c r="N25" s="4" t="str">
+        <x:v>P3-T04</x:v>
+      </x:c>
+      <x:c r="O25" s="4" t="str">
+        <x:v>Assembler/CKD validation</x:v>
+      </x:c>
+      <x:c r="P25" s="4" t="str">
+        <x:v>No public contact or engine fit verified</x:v>
+      </x:c>
+      <x:c r="Q25" s="4" t="str">
+        <x:v>Medium</x:v>
+      </x:c>
+      <x:c r="R25" s="4" t="str">
+        <x:v>NOT CONTACTED</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="4" t="str">
+        <x:v>Tanzania</x:v>
+      </x:c>
+      <x:c r="B26" s="4" t="str">
+        <x:v>CRSG Tanzania Trading Co Ltd</x:v>
+      </x:c>
+      <x:c r="C26" s="4" t="str">
+        <x:v>CKD beneficiary candidate</x:v>
+      </x:c>
+      <x:c r="D26" s="4" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="E26" s="4" t="str">
+        <x:v>Motorcycle/tricycle CKD</x:v>
+      </x:c>
+      <x:c r="F26" s="4" t="str">
+        <x:v>EAC duty-remission listing</x:v>
+      </x:c>
+      <x:c r="G26" s="4" t="str">
+        <x:v>https://www.eac.int/documents?controller=download&amp;file=6c5739ac-842c-43bc-96be-1cd168ed415f&amp;name=EAC+Vol+AT+1+NO+29+SEPTEMBER+2025.pdf&amp;task=download.file</x:v>
+      </x:c>
+      <x:c r="H26" s="4" t="str"/>
+      <x:c r="I26" s="4" t="str"/>
+      <x:c r="J26" s="4" t="str"/>
+      <x:c r="K26" s="4" t="str"/>
+      <x:c r="L26" s="4" t="str">
+        <x:v>Tanzania</x:v>
+      </x:c>
+      <x:c r="M26" s="4" t="str">
+        <x:v>NOT VERIFIED</x:v>
+      </x:c>
+      <x:c r="N26" s="4" t="str">
+        <x:v>P3-T04</x:v>
+      </x:c>
+      <x:c r="O26" s="4" t="str">
+        <x:v>Assembler/CKD validation</x:v>
+      </x:c>
+      <x:c r="P26" s="4" t="str">
+        <x:v>No public contact or engine fit verified</x:v>
+      </x:c>
+      <x:c r="Q26" s="4" t="str">
+        <x:v>Medium</x:v>
+      </x:c>
+      <x:c r="R26" s="4" t="str">
+        <x:v>NOT CONTACTED</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" s="4" t="str">
+        <x:v>Tanzania</x:v>
+      </x:c>
+      <x:c r="B27" s="4" t="str">
+        <x:v>Kishan Enterprises Ltd</x:v>
+      </x:c>
+      <x:c r="C27" s="4" t="str">
+        <x:v>CKD beneficiary candidate</x:v>
+      </x:c>
+      <x:c r="D27" s="4" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="E27" s="4" t="str">
+        <x:v>Motorcycle/tricycle CKD</x:v>
+      </x:c>
+      <x:c r="F27" s="4" t="str">
+        <x:v>EAC duty-remission listing</x:v>
+      </x:c>
+      <x:c r="G27" s="4" t="str">
+        <x:v>https://www.eac.int/documents?controller=download&amp;file=6c5739ac-842c-43bc-96be-1cd168ed415f&amp;name=EAC+Vol+AT+1+NO+29+SEPTEMBER+2025.pdf&amp;task=download.file</x:v>
+      </x:c>
+      <x:c r="H27" s="4" t="str"/>
+      <x:c r="I27" s="4" t="str"/>
+      <x:c r="J27" s="4" t="str"/>
+      <x:c r="K27" s="4" t="str"/>
+      <x:c r="L27" s="4" t="str">
+        <x:v>Tanzania</x:v>
+      </x:c>
+      <x:c r="M27" s="4" t="str">
+        <x:v>NOT VERIFIED</x:v>
+      </x:c>
+      <x:c r="N27" s="4" t="str">
+        <x:v>P3-T04</x:v>
+      </x:c>
+      <x:c r="O27" s="4" t="str">
+        <x:v>Assembler/CKD validation</x:v>
+      </x:c>
+      <x:c r="P27" s="4" t="str">
+        <x:v>No public contact or engine fit verified</x:v>
+      </x:c>
+      <x:c r="Q27" s="4" t="str">
+        <x:v>Medium</x:v>
+      </x:c>
+      <x:c r="R27" s="4" t="str">
+        <x:v>NOT CONTACTED</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" s="4" t="str">
+        <x:v>Tanzania</x:v>
+      </x:c>
+      <x:c r="B28" s="4" t="str">
+        <x:v>Sulong Motors Co Ltd</x:v>
+      </x:c>
+      <x:c r="C28" s="4" t="str">
+        <x:v>CKD beneficiary candidate</x:v>
+      </x:c>
+      <x:c r="D28" s="4" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="E28" s="4" t="str">
+        <x:v>Motorcycle/tricycle CKD</x:v>
+      </x:c>
+      <x:c r="F28" s="4" t="str">
+        <x:v>EAC duty-remission listing</x:v>
+      </x:c>
+      <x:c r="G28" s="4" t="str">
+        <x:v>https://www.eac.int/documents?controller=download&amp;file=6c5739ac-842c-43bc-96be-1cd168ed415f&amp;name=EAC+Vol+AT+1+NO+29+SEPTEMBER+2025.pdf&amp;task=download.file</x:v>
+      </x:c>
+      <x:c r="H28" s="4" t="str"/>
+      <x:c r="I28" s="4" t="str"/>
+      <x:c r="J28" s="4" t="str"/>
+      <x:c r="K28" s="4" t="str"/>
+      <x:c r="L28" s="4" t="str">
+        <x:v>Tanzania</x:v>
+      </x:c>
+      <x:c r="M28" s="4" t="str">
+        <x:v>NOT VERIFIED</x:v>
+      </x:c>
+      <x:c r="N28" s="4" t="str">
+        <x:v>P3-T04</x:v>
+      </x:c>
+      <x:c r="O28" s="4" t="str">
+        <x:v>Assembler/CKD validation</x:v>
+      </x:c>
+      <x:c r="P28" s="4" t="str">
+        <x:v>No public contact or engine fit verified</x:v>
+      </x:c>
+      <x:c r="Q28" s="4" t="str">
+        <x:v>Medium</x:v>
+      </x:c>
+      <x:c r="R28" s="4" t="str">
+        <x:v>NOT CONTACTED</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" s="4" t="str">
+        <x:v>Tanzania</x:v>
+      </x:c>
+      <x:c r="B29" s="4" t="str">
+        <x:v>Carter Investment Co Ltd</x:v>
+      </x:c>
+      <x:c r="C29" s="4" t="str">
+        <x:v>CKD beneficiary candidate</x:v>
+      </x:c>
+      <x:c r="D29" s="4" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="E29" s="4" t="str">
+        <x:v>Motorcycle/tricycle CKD</x:v>
+      </x:c>
+      <x:c r="F29" s="4" t="str">
+        <x:v>EAC duty-remission listing</x:v>
+      </x:c>
+      <x:c r="G29" s="4" t="str">
+        <x:v>https://www.eac.int/documents?controller=download&amp;file=6c5739ac-842c-43bc-96be-1cd168ed415f&amp;name=EAC+Vol+AT+1+NO+29+SEPTEMBER+2025.pdf&amp;task=download.file</x:v>
+      </x:c>
+      <x:c r="H29" s="4" t="str"/>
+      <x:c r="I29" s="4" t="str"/>
+      <x:c r="J29" s="4" t="str"/>
+      <x:c r="K29" s="4" t="str"/>
+      <x:c r="L29" s="4" t="str">
+        <x:v>Tanzania</x:v>
+      </x:c>
+      <x:c r="M29" s="4" t="str">
+        <x:v>NOT VERIFIED</x:v>
+      </x:c>
+      <x:c r="N29" s="4" t="str">
+        <x:v>P3-T04</x:v>
+      </x:c>
+      <x:c r="O29" s="4" t="str">
+        <x:v>Assembler/CKD validation</x:v>
+      </x:c>
+      <x:c r="P29" s="4" t="str">
+        <x:v>No public contact or engine fit verified</x:v>
+      </x:c>
+      <x:c r="Q29" s="4" t="str">
+        <x:v>Medium</x:v>
+      </x:c>
+      <x:c r="R29" s="4" t="str">
+        <x:v>NOT CONTACTED</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" s="4" t="str">
+        <x:v>Tanzania</x:v>
+      </x:c>
+      <x:c r="B30" s="4" t="str">
+        <x:v>KWM Motors Tanzania Ltd</x:v>
+      </x:c>
+      <x:c r="C30" s="4" t="str">
+        <x:v>CKD beneficiary candidate</x:v>
+      </x:c>
+      <x:c r="D30" s="4" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="E30" s="4" t="str">
+        <x:v>Motorcycle/tricycle CKD</x:v>
+      </x:c>
+      <x:c r="F30" s="4" t="str">
+        <x:v>EAC duty-remission listing</x:v>
+      </x:c>
+      <x:c r="G30" s="4" t="str">
+        <x:v>https://www.eac.int/documents?controller=download&amp;file=6c5739ac-842c-43bc-96be-1cd168ed415f&amp;name=EAC+Vol+AT+1+NO+29+SEPTEMBER+2025.pdf&amp;task=download.file</x:v>
+      </x:c>
+      <x:c r="H30" s="4" t="str"/>
+      <x:c r="I30" s="4" t="str"/>
+      <x:c r="J30" s="4" t="str"/>
+      <x:c r="K30" s="4" t="str"/>
+      <x:c r="L30" s="4" t="str">
+        <x:v>Tanzania</x:v>
+      </x:c>
+      <x:c r="M30" s="4" t="str">
+        <x:v>NOT VERIFIED</x:v>
+      </x:c>
+      <x:c r="N30" s="4" t="str">
+        <x:v>P3-T04</x:v>
+      </x:c>
+      <x:c r="O30" s="4" t="str">
+        <x:v>Assembler/CKD validation</x:v>
+      </x:c>
+      <x:c r="P30" s="4" t="str">
+        <x:v>No public contact or engine fit verified</x:v>
+      </x:c>
+      <x:c r="Q30" s="4" t="str">
+        <x:v>Medium</x:v>
+      </x:c>
+      <x:c r="R30" s="4" t="str">
+        <x:v>NOT CONTACTED</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31">
+      <x:c r="A31" s="4" t="str">
+        <x:v>Tanzania</x:v>
+      </x:c>
+      <x:c r="B31" s="4" t="str">
+        <x:v>SanLG Tanzania Ltd</x:v>
+      </x:c>
+      <x:c r="C31" s="4" t="str">
+        <x:v>CKD beneficiary candidate</x:v>
+      </x:c>
+      <x:c r="D31" s="4" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="E31" s="4" t="str">
+        <x:v>Motorcycle/tricycle CKD</x:v>
+      </x:c>
+      <x:c r="F31" s="4" t="str">
+        <x:v>EAC duty-remission listing</x:v>
+      </x:c>
+      <x:c r="G31" s="4" t="str">
+        <x:v>https://www.eac.int/documents?controller=download&amp;file=6c5739ac-842c-43bc-96be-1cd168ed415f&amp;name=EAC+Vol+AT+1+NO+29+SEPTEMBER+2025.pdf&amp;task=download.file</x:v>
+      </x:c>
+      <x:c r="H31" s="4" t="str"/>
+      <x:c r="I31" s="4" t="str"/>
+      <x:c r="J31" s="4" t="str"/>
+      <x:c r="K31" s="4" t="str"/>
+      <x:c r="L31" s="4" t="str">
+        <x:v>Tanzania</x:v>
+      </x:c>
+      <x:c r="M31" s="4" t="str">
+        <x:v>NOT VERIFIED</x:v>
+      </x:c>
+      <x:c r="N31" s="4" t="str">
+        <x:v>P3-T04</x:v>
+      </x:c>
+      <x:c r="O31" s="4" t="str">
+        <x:v>Assembler/CKD validation</x:v>
+      </x:c>
+      <x:c r="P31" s="4" t="str">
+        <x:v>No public contact or engine fit verified</x:v>
+      </x:c>
+      <x:c r="Q31" s="4" t="str">
+        <x:v>Medium</x:v>
+      </x:c>
+      <x:c r="R31" s="4" t="str">
+        <x:v>NOT CONTACTED</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32">
+      <x:c r="A32" s="4" t="str">
+        <x:v>Tanzania</x:v>
+      </x:c>
+      <x:c r="B32" s="4" t="str">
+        <x:v>Shiv Sai Ltd</x:v>
+      </x:c>
+      <x:c r="C32" s="4" t="str">
+        <x:v>CKD beneficiary candidate</x:v>
+      </x:c>
+      <x:c r="D32" s="4" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="E32" s="4" t="str">
+        <x:v>Motorcycle/tricycle CKD</x:v>
+      </x:c>
+      <x:c r="F32" s="4" t="str">
+        <x:v>EAC duty-remission listing</x:v>
+      </x:c>
+      <x:c r="G32" s="4" t="str">
+        <x:v>https://www.eac.int/documents?controller=download&amp;file=6c5739ac-842c-43bc-96be-1cd168ed415f&amp;name=EAC+Vol+AT+1+NO+29+SEPTEMBER+2025.pdf&amp;task=download.file</x:v>
+      </x:c>
+      <x:c r="H32" s="4" t="str"/>
+      <x:c r="I32" s="4" t="str"/>
+      <x:c r="J32" s="4" t="str"/>
+      <x:c r="K32" s="4" t="str"/>
+      <x:c r="L32" s="4" t="str">
+        <x:v>Tanzania</x:v>
+      </x:c>
+      <x:c r="M32" s="4" t="str">
+        <x:v>NOT VERIFIED</x:v>
+      </x:c>
+      <x:c r="N32" s="4" t="str">
+        <x:v>P3-T04</x:v>
+      </x:c>
+      <x:c r="O32" s="4" t="str">
+        <x:v>Assembler/CKD validation</x:v>
+      </x:c>
+      <x:c r="P32" s="4" t="str">
+        <x:v>No public contact or engine fit verified</x:v>
+      </x:c>
+      <x:c r="Q32" s="4" t="str">
+        <x:v>Medium</x:v>
+      </x:c>
+      <x:c r="R32" s="4" t="str">
+        <x:v>NOT CONTACTED</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33">
+      <x:c r="A33" s="4" t="str">
+        <x:v>Tanzania</x:v>
+      </x:c>
+      <x:c r="B33" s="4" t="str">
+        <x:v>Shinyanga Emporium (1978) Ltd</x:v>
+      </x:c>
+      <x:c r="C33" s="4" t="str">
+        <x:v>CKD beneficiary candidate</x:v>
+      </x:c>
+      <x:c r="D33" s="4" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="E33" s="4" t="str">
+        <x:v>Motorcycle/tricycle CKD</x:v>
+      </x:c>
+      <x:c r="F33" s="4" t="str">
+        <x:v>EAC duty-remission listing</x:v>
+      </x:c>
+      <x:c r="G33" s="4" t="str">
+        <x:v>https://www.eac.int/documents?controller=download&amp;file=6c5739ac-842c-43bc-96be-1cd168ed415f&amp;name=EAC+Vol+AT+1+NO+29+SEPTEMBER+2025.pdf&amp;task=download.file</x:v>
+      </x:c>
+      <x:c r="H33" s="4" t="str"/>
+      <x:c r="I33" s="4" t="str"/>
+      <x:c r="J33" s="4" t="str"/>
+      <x:c r="K33" s="4" t="str"/>
+      <x:c r="L33" s="4" t="str">
+        <x:v>Tanzania</x:v>
+      </x:c>
+      <x:c r="M33" s="4" t="str">
+        <x:v>NOT VERIFIED</x:v>
+      </x:c>
+      <x:c r="N33" s="4" t="str">
+        <x:v>P3-T04</x:v>
+      </x:c>
+      <x:c r="O33" s="4" t="str">
+        <x:v>Assembler/CKD validation</x:v>
+      </x:c>
+      <x:c r="P33" s="4" t="str">
+        <x:v>No public contact or engine fit verified</x:v>
+      </x:c>
+      <x:c r="Q33" s="4" t="str">
+        <x:v>Medium</x:v>
+      </x:c>
+      <x:c r="R33" s="4" t="str">
+        <x:v>NOT CONTACTED</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34">
+      <x:c r="A34" s="4" t="str">
+        <x:v>Tanzania</x:v>
+      </x:c>
+      <x:c r="B34" s="4" t="str">
+        <x:v>Masway Co Ltd</x:v>
+      </x:c>
+      <x:c r="C34" s="4" t="str">
+        <x:v>CKD beneficiary candidate</x:v>
+      </x:c>
+      <x:c r="D34" s="4" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="E34" s="4" t="str">
+        <x:v>Motorcycle/tricycle CKD</x:v>
+      </x:c>
+      <x:c r="F34" s="4" t="str">
+        <x:v>EAC duty-remission listing</x:v>
+      </x:c>
+      <x:c r="G34" s="4" t="str">
+        <x:v>https://www.eac.int/documents?controller=download&amp;file=6c5739ac-842c-43bc-96be-1cd168ed415f&amp;name=EAC+Vol+AT+1+NO+29+SEPTEMBER+2025.pdf&amp;task=download.file</x:v>
+      </x:c>
+      <x:c r="H34" s="4" t="str"/>
+      <x:c r="I34" s="4" t="str"/>
+      <x:c r="J34" s="4" t="str"/>
+      <x:c r="K34" s="4" t="str"/>
+      <x:c r="L34" s="4" t="str">
+        <x:v>Tanzania</x:v>
+      </x:c>
+      <x:c r="M34" s="4" t="str">
+        <x:v>NOT VERIFIED</x:v>
+      </x:c>
+      <x:c r="N34" s="4" t="str">
+        <x:v>P3-T04</x:v>
+      </x:c>
+      <x:c r="O34" s="4" t="str">
+        <x:v>Assembler/CKD validation</x:v>
+      </x:c>
+      <x:c r="P34" s="4" t="str">
+        <x:v>No public contact or engine fit verified</x:v>
+      </x:c>
+      <x:c r="Q34" s="4" t="str">
+        <x:v>Medium</x:v>
+      </x:c>
+      <x:c r="R34" s="4" t="str">
+        <x:v>NOT CONTACTED</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35">
+      <x:c r="A35" s="4" t="str">
+        <x:v>Tanzania</x:v>
+      </x:c>
+      <x:c r="B35" s="4" t="str">
+        <x:v>SanLG Worldwide Investment Ltd</x:v>
+      </x:c>
+      <x:c r="C35" s="4" t="str">
+        <x:v>CKD beneficiary candidate</x:v>
+      </x:c>
+      <x:c r="D35" s="4" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="E35" s="4" t="str">
+        <x:v>Motorcycle/tricycle CKD</x:v>
+      </x:c>
+      <x:c r="F35" s="4" t="str">
+        <x:v>EAC duty-remission listing</x:v>
+      </x:c>
+      <x:c r="G35" s="4" t="str">
+        <x:v>https://www.eac.int/documents?controller=download&amp;file=6c5739ac-842c-43bc-96be-1cd168ed415f&amp;name=EAC+Vol+AT+1+NO+29+SEPTEMBER+2025.pdf&amp;task=download.file</x:v>
+      </x:c>
+      <x:c r="H35" s="4" t="str"/>
+      <x:c r="I35" s="4" t="str"/>
+      <x:c r="J35" s="4" t="str"/>
+      <x:c r="K35" s="4" t="str"/>
+      <x:c r="L35" s="4" t="str">
+        <x:v>Tanzania</x:v>
+      </x:c>
+      <x:c r="M35" s="4" t="str">
+        <x:v>NOT VERIFIED</x:v>
+      </x:c>
+      <x:c r="N35" s="4" t="str">
+        <x:v>P3-T04</x:v>
+      </x:c>
+      <x:c r="O35" s="4" t="str">
+        <x:v>Assembler/CKD validation</x:v>
+      </x:c>
+      <x:c r="P35" s="4" t="str">
+        <x:v>No public contact or engine fit verified</x:v>
+      </x:c>
+      <x:c r="Q35" s="4" t="str">
+        <x:v>Medium</x:v>
+      </x:c>
+      <x:c r="R35" s="4" t="str">
+        <x:v>NOT CONTACTED</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36">
+      <x:c r="A36" s="4" t="str">
+        <x:v>Uzbekistan</x:v>
+      </x:c>
+      <x:c r="B36" s="4" t="str">
+        <x:v>Bikeland</x:v>
+      </x:c>
+      <x:c r="C36" s="4" t="str">
+        <x:v>Retailer/service</x:v>
+      </x:c>
+      <x:c r="D36" s="4" t="str">
+        <x:v>Lifan; Zongshen</x:v>
+      </x:c>
+      <x:c r="E36" s="4" t="str">
+        <x:v>Motorcycles; tricycles; engines; parts</x:v>
+      </x:c>
+      <x:c r="F36" s="4" t="str">
+        <x:v>Website listing</x:v>
+      </x:c>
+      <x:c r="G36" s="4" t="str">
+        <x:v>https://www.bikeland.uz/</x:v>
+      </x:c>
+      <x:c r="H36" s="4" t="str"/>
+      <x:c r="I36" s="4" t="str">
+        <x:v>info@bikeland.uz</x:v>
+      </x:c>
+      <x:c r="J36" s="4" t="str">
+        <x:v>+998555006001</x:v>
+      </x:c>
+      <x:c r="K36" s="4" t="str"/>
+      <x:c r="L36" s="4" t="str">
+        <x:v>Tashkent</x:v>
+      </x:c>
+      <x:c r="M36" s="4" t="str">
+        <x:v>Public email/phone</x:v>
+      </x:c>
+      <x:c r="N36" s="4" t="str">
+        <x:v>P3-U01</x:v>
+      </x:c>
+      <x:c r="O36" s="4" t="str">
+        <x:v>Accelerated validation</x:v>
+      </x:c>
+      <x:c r="P36" s="4" t="str">
+        <x:v>Retailer not national wholesaler</x:v>
+      </x:c>
+      <x:c r="Q36" s="4" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="R36" s="4" t="str">
+        <x:v>NOT CONTACTED</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37">
+      <x:c r="A37" s="4" t="str">
+        <x:v>Uzbekistan</x:v>
+      </x:c>
+      <x:c r="B37" s="4" t="str">
+        <x:v>Hadid Moto</x:v>
+      </x:c>
+      <x:c r="C37" s="4" t="str">
+        <x:v>Parts supplier</x:v>
+      </x:c>
+      <x:c r="D37" s="4" t="str">
+        <x:v>Various</x:v>
+      </x:c>
+      <x:c r="E37" s="4" t="str">
+        <x:v>Motorcycle parts</x:v>
+      </x:c>
+      <x:c r="F37" s="4" t="str">
+        <x:v>Company website</x:v>
+      </x:c>
+      <x:c r="G37" s="4" t="str">
+        <x:v>https://hadidmoto.uz/</x:v>
+      </x:c>
+      <x:c r="H37" s="4" t="str"/>
+      <x:c r="I37" s="4" t="str">
+        <x:v>HadidMoto@store.com</x:v>
+      </x:c>
+      <x:c r="J37" s="4" t="str">
+        <x:v>+998904045555</x:v>
+      </x:c>
+      <x:c r="K37" s="4" t="str"/>
+      <x:c r="L37" s="4" t="str">
+        <x:v>Fergana</x:v>
+      </x:c>
+      <x:c r="M37" s="4" t="str">
+        <x:v>Public email/phone</x:v>
+      </x:c>
+      <x:c r="N37" s="4" t="str">
+        <x:v>P3-U03</x:v>
+      </x:c>
+      <x:c r="O37" s="4" t="str">
+        <x:v>Parts channel</x:v>
+      </x:c>
+      <x:c r="P37" s="4" t="str">
+        <x:v>Parts-only evidence</x:v>
+      </x:c>
+      <x:c r="Q37" s="4" t="str">
+        <x:v>Medium</x:v>
+      </x:c>
+      <x:c r="R37" s="4" t="str">
+        <x:v>NOT CONTACTED</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38">
+      <x:c r="A38" s="4" t="str">
+        <x:v>Uzbekistan</x:v>
+      </x:c>
+      <x:c r="B38" s="4" t="str">
+        <x:v>CFMOTO Uzbekistan</x:v>
+      </x:c>
+      <x:c r="C38" s="4" t="str">
+        <x:v>Official distributor</x:v>
+      </x:c>
+      <x:c r="D38" s="4" t="str">
+        <x:v>CFMOTO</x:v>
+      </x:c>
+      <x:c r="E38" s="4" t="str">
+        <x:v>Motorcycles</x:v>
+      </x:c>
+      <x:c r="F38" s="4" t="str">
+        <x:v>Official distributor</x:v>
+      </x:c>
+      <x:c r="G38" s="4" t="str">
+        <x:v>https://cfmoto.uz/</x:v>
+      </x:c>
+      <x:c r="H38" s="4" t="str"/>
+      <x:c r="I38" s="4" t="str"/>
+      <x:c r="J38" s="4" t="str"/>
+      <x:c r="K38" s="4" t="str"/>
+      <x:c r="L38" s="4" t="str">
+        <x:v>Uzbekistan</x:v>
+      </x:c>
+      <x:c r="M38" s="4" t="str">
+        <x:v>Public company route</x:v>
+      </x:c>
+      <x:c r="N38" s="4" t="str">
+        <x:v>P3-U04</x:v>
+      </x:c>
+      <x:c r="O38" s="4" t="str">
+        <x:v>Channel mapping</x:v>
+      </x:c>
+      <x:c r="P38" s="4" t="str">
+        <x:v>Separate platform; no fit inferred</x:v>
+      </x:c>
+      <x:c r="Q38" s="4" t="str">
+        <x:v>Medium</x:v>
+      </x:c>
+      <x:c r="R38" s="4" t="str">
+        <x:v>NOT CONTACTED</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39">
+      <x:c r="A39" s="4" t="str">
         <x:v>Russia</x:v>
       </x:c>
-      <x:c r="M10" s="4" t="str">
+      <x:c r="B39" s="4" t="str">
+        <x:v>Loncin Russia</x:v>
+      </x:c>
+      <x:c r="C39" s="4" t="str">
+        <x:v>Official representative</x:v>
+      </x:c>
+      <x:c r="D39" s="4" t="str">
+        <x:v>Loncin</x:v>
+      </x:c>
+      <x:c r="E39" s="4" t="str">
+        <x:v>Motorcycles/parts</x:v>
+      </x:c>
+      <x:c r="F39" s="4" t="str">
+        <x:v>Representative page</x:v>
+      </x:c>
+      <x:c r="G39" s="4" t="str">
+        <x:v>https://loncin.pro/company</x:v>
+      </x:c>
+      <x:c r="H39" s="4" t="str"/>
+      <x:c r="I39" s="4" t="str"/>
+      <x:c r="J39" s="4" t="str"/>
+      <x:c r="K39" s="4" t="str"/>
+      <x:c r="L39" s="4" t="str">
+        <x:v>Russia</x:v>
+      </x:c>
+      <x:c r="M39" s="4" t="str">
         <x:v>Public company route</x:v>
       </x:c>
-      <x:c r="N10" s="4" t="str">
+      <x:c r="N39" s="4" t="str">
+        <x:v>P3-R01</x:v>
+      </x:c>
+      <x:c r="O39" s="4" t="str">
+        <x:v>Distributor mapping</x:v>
+      </x:c>
+      <x:c r="P39" s="4" t="str">
+        <x:v>Compliance unresolved</x:v>
+      </x:c>
+      <x:c r="Q39" s="4" t="str">
+        <x:v>Medium</x:v>
+      </x:c>
+      <x:c r="R39" s="4" t="str">
+        <x:v>NOT CONTACTED</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40">
+      <x:c r="A40" s="4" t="str">
+        <x:v>Russia</x:v>
+      </x:c>
+      <x:c r="B40" s="4" t="str">
+        <x:v>Lifan Russia</x:v>
+      </x:c>
+      <x:c r="C40" s="4" t="str">
+        <x:v>Official representative</x:v>
+      </x:c>
+      <x:c r="D40" s="4" t="str">
+        <x:v>Lifan</x:v>
+      </x:c>
+      <x:c r="E40" s="4" t="str">
+        <x:v>Motorcycles/parts</x:v>
+      </x:c>
+      <x:c r="F40" s="4" t="str">
+        <x:v>Representative page</x:v>
+      </x:c>
+      <x:c r="G40" s="4" t="str">
+        <x:v>https://lifan-moto.ru/</x:v>
+      </x:c>
+      <x:c r="H40" s="4" t="str"/>
+      <x:c r="I40" s="4" t="str"/>
+      <x:c r="J40" s="4" t="str"/>
+      <x:c r="K40" s="4" t="str"/>
+      <x:c r="L40" s="4" t="str">
+        <x:v>Russia</x:v>
+      </x:c>
+      <x:c r="M40" s="4" t="str">
+        <x:v>Public company route</x:v>
+      </x:c>
+      <x:c r="N40" s="4" t="str">
         <x:v>P3-R02</x:v>
       </x:c>
-      <x:c r="O10" s="4" t="str">
+      <x:c r="O40" s="4" t="str">
         <x:v>Distributor mapping</x:v>
       </x:c>
-      <x:c r="P10" s="4" t="str">
+      <x:c r="P40" s="4" t="str">
         <x:v>Compliance unresolved</x:v>
       </x:c>
-      <x:c r="Q10" s="4" t="str">
-        <x:v>Medium</x:v>
-      </x:c>
-      <x:c r="R10" s="4" t="str">
+      <x:c r="Q40" s="4" t="str">
+        <x:v>Medium</x:v>
+      </x:c>
+      <x:c r="R40" s="4" t="str">
+        <x:v>NOT CONTACTED</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41">
+      <x:c r="A41" s="4" t="str">
+        <x:v>Colombia</x:v>
+      </x:c>
+      <x:c r="B41" s="4" t="str">
+        <x:v>CG200/250 parts marketplace sellers</x:v>
+      </x:c>
+      <x:c r="C41" s="4" t="str">
+        <x:v>Marketplace seller</x:v>
+      </x:c>
+      <x:c r="D41" s="4" t="str">
+        <x:v>Zongshen; Loncin; CG</x:v>
+      </x:c>
+      <x:c r="E41" s="4" t="str">
+        <x:v>Starter part</x:v>
+      </x:c>
+      <x:c r="F41" s="4" t="str">
+        <x:v>Parts listing</x:v>
+      </x:c>
+      <x:c r="G41" s="4" t="str">
+        <x:v>https://articulo.mercadolibre.com.co/MCO-3530541364-motor-de-arranque-para-zongshen-loncin-cg200-cg250-_JM</x:v>
+      </x:c>
+      <x:c r="H41" s="4" t="str"/>
+      <x:c r="I41" s="4" t="str"/>
+      <x:c r="J41" s="4" t="str"/>
+      <x:c r="K41" s="4" t="str"/>
+      <x:c r="L41" s="4" t="str">
+        <x:v>Colombia</x:v>
+      </x:c>
+      <x:c r="M41" s="4" t="str">
+        <x:v>NOT B2B VERIFIED</x:v>
+      </x:c>
+      <x:c r="N41" s="4" t="str">
+        <x:v>P3-C02</x:v>
+      </x:c>
+      <x:c r="O41" s="4" t="str">
+        <x:v>Only a research lead</x:v>
+      </x:c>
+      <x:c r="P41" s="4" t="str">
+        <x:v>Parts-only; not buyer or engine demand</x:v>
+      </x:c>
+      <x:c r="Q41" s="4" t="str">
+        <x:v>Low</x:v>
+      </x:c>
+      <x:c r="R41" s="4" t="str">
         <x:v>NOT CONTACTED</x:v>
       </x:c>
     </x:row>

</xml_diff>